<commit_message>
Add ErrorHandling Skills; Validate ColInfo class
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/tests/test_data/ColInfo.xlsx
+++ b/tests/test_data/ColInfo.xlsx
@@ -5,16 +5,27 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Box Sync\Projects\Excel_Steps\tests\test_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Library\CloudStorage\Box-Box\Projects\Excel_Steps\tests\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76F5808-FACF-4359-B950-096B3A4985CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EE6B64-16FE-4B6B-9DFF-76F3341A3425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3675" yWindow="503" windowWidth="26017" windowHeight="15697" xr2:uid="{CF177DA8-F40C-4AC0-BFD2-2712428C7C73}"/>
+    <workbookView xWindow="13800" yWindow="2618" windowWidth="16567" windowHeight="10709" xr2:uid="{CF177DA8-F40C-4AC0-BFD2-2712428C7C73}"/>
   </bookViews>
   <sheets>
     <sheet name="colinfo_" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="BR_Example">colinfo_!$G:$G</definedName>
+    <definedName name="data_type_VBA">colinfo_!$F:$F</definedName>
+    <definedName name="Description">colinfo_!$D:$D</definedName>
+    <definedName name="IsIndex">colinfo_!$C:$C</definedName>
+    <definedName name="rand">colinfo_!$I:$I</definedName>
+    <definedName name="Second_Tbl">colinfo_!$H:$H</definedName>
+    <definedName name="units">colinfo_!$E:$E</definedName>
+    <definedName name="VarNameNorm">colinfo_!$A:$A</definedName>
+    <definedName name="VarNameRaw">colinfo_!$B:$B</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -749,322 +760,320 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="3">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G2" s="4"/>
-      <c r="H2">
+      <c r="D2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="4">
         <v>1</v>
       </c>
       <c r="I2" s="6">
         <f ca="1">RAND()</f>
-        <v>0.91452069972924077</v>
+        <v>0.71260211605019719</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" s="4"/>
-      <c r="H3">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="4">
         <v>2</v>
       </c>
       <c r="I3" s="6">
-        <f t="shared" ref="I3:I14" ca="1" si="0">RAND()</f>
-        <v>0.60543921123433642</v>
+        <f ca="1">RAND()</f>
+        <v>7.3976576902260893E-2</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A4" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4">
+      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="4">
         <v>3</v>
       </c>
       <c r="I4" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.4849948982726372</v>
+        <f ca="1">RAND()</f>
+        <v>0.94134841982711548</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A5" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="4">
         <v>4</v>
       </c>
       <c r="I5" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.15098342785265828</v>
+        <f ca="1">RAND()</f>
+        <v>0.62868725250687318</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="4">
-        <v>1</v>
-      </c>
       <c r="I6" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.48587210281363902</v>
+        <f ca="1">RAND()</f>
+        <v>0.84005428459187781</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="4">
-        <v>2</v>
-      </c>
       <c r="I7" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.64505592927690192</v>
+        <f ca="1">RAND()</f>
+        <v>2.7874064624666905E-2</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="4">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G8" s="4">
-        <v>3</v>
-      </c>
       <c r="I8" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.15660356601166647</v>
+        <f ca="1">RAND()</f>
+        <v>0.91536273521502443</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="4">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G9" s="4">
-        <v>4</v>
-      </c>
       <c r="I9" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.27196465670111802</v>
+        <f ca="1">RAND()</f>
+        <v>0.71506805238535442</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A10" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>47</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I10" s="6">
+        <f ca="1">RAND()</f>
+        <v>0.29431600334252406</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G11" s="4"/>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11" s="6">
+        <f ca="1">RAND()</f>
+        <v>0.93016278882487313</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12">
+        <v>4</v>
+      </c>
+      <c r="I12" s="6">
+        <f ca="1">RAND()</f>
+        <v>0.36342056568959991</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G10" s="4">
-        <v>5</v>
-      </c>
-      <c r="I10" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.39178072898392191</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G11" s="4">
-        <v>6</v>
-      </c>
-      <c r="I11" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.24351029927926227</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G12" s="4">
-        <v>7</v>
-      </c>
-      <c r="I12" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.68413865024278653</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G13" s="4">
-        <v>8</v>
+      <c r="G13" s="4"/>
+      <c r="H13">
+        <v>2</v>
       </c>
       <c r="I13" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.96597652971422887</v>
+        <f ca="1">RAND()</f>
+        <v>7.8645057123848394E-3</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>31</v>
+      <c r="A14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="H14">
+        <v>3</v>
       </c>
       <c r="I14" s="6">
-        <f t="shared" ca="1" si="0"/>
-        <v>0.4351324487641921</v>
+        <f ca="1">RAND()</f>
+        <v>0.61530357197018049</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test_data/ColInfo.xlsx updates for upcoming Change_
</commit_message>
<xml_diff>
--- a/tests/test_data/ColInfo.xlsx
+++ b/tests/test_data/ColInfo.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Library\CloudStorage\Box-Box\Projects\Excel_Steps\tests\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EE6B64-16FE-4B6B-9DFF-76F3341A3425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1395CBF-8BE5-455B-A74A-C788532753F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13800" yWindow="2618" windowWidth="16567" windowHeight="10709" xr2:uid="{CF177DA8-F40C-4AC0-BFD2-2712428C7C73}"/>
+    <workbookView xWindow="368" yWindow="368" windowWidth="16567" windowHeight="10710" xr2:uid="{CF177DA8-F40C-4AC0-BFD2-2712428C7C73}"/>
   </bookViews>
   <sheets>
     <sheet name="colinfo_" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="BR_Example">colinfo_!$G:$G</definedName>
+    <definedName name="BR_Example">colinfo_!$I:$I</definedName>
     <definedName name="data_type_VBA">colinfo_!$F:$F</definedName>
     <definedName name="Description">colinfo_!$D:$D</definedName>
     <definedName name="IsIndex">colinfo_!$C:$C</definedName>
-    <definedName name="rand">colinfo_!$I:$I</definedName>
-    <definedName name="Second_Tbl">colinfo_!$H:$H</definedName>
+    <definedName name="rand">colinfo_!$K:$K</definedName>
+    <definedName name="Second_Tbl">colinfo_!$J:$J</definedName>
     <definedName name="units">colinfo_!$E:$E</definedName>
     <definedName name="VarNameNorm">colinfo_!$A:$A</definedName>
     <definedName name="VarNameRaw">colinfo_!$B:$B</definedName>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="57">
   <si>
     <t>Description</t>
   </si>
@@ -209,6 +209,18 @@
   </si>
   <si>
     <t>rand</t>
+  </si>
+  <si>
+    <t>FillVals</t>
+  </si>
+  <si>
+    <t>{BLANK:Unknown,Locn10:Locn1}</t>
+  </si>
+  <si>
+    <t>FilterVals</t>
+  </si>
+  <si>
+    <t>{KeepOnly:Online}</t>
   </si>
 </sst>
 </file>
@@ -717,7 +729,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D8961A3-90B8-45BB-ADA5-B09F327CFDF3}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.53125" bestFit="1" customWidth="1"/>
@@ -726,11 +738,13 @@
     <col min="4" max="4" width="20.06640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.19921875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.796875" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -749,17 +763,23 @@
       <c r="F1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="I1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -776,15 +796,19 @@
       <c r="F2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="I2" s="4">
         <v>1</v>
       </c>
-      <c r="I2" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.71260211605019719</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K2" s="6">
+        <f t="shared" ref="K2:K14" ca="1" si="0">RAND()</f>
+        <v>0.83141208391015298</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -801,15 +825,19 @@
       <c r="F3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="4">
         <v>2</v>
       </c>
-      <c r="I3" s="6">
-        <f ca="1">RAND()</f>
-        <v>7.3976576902260893E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K3" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.65216747104172024</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -826,15 +854,17 @@
       <c r="F4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="4">
         <v>3</v>
       </c>
-      <c r="I4" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.94134841982711548</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K4" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.21351277071252484</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -851,15 +881,17 @@
       <c r="F5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="4">
         <v>4</v>
       </c>
-      <c r="I5" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.62868725250687318</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K5" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.80748944699456604</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -876,15 +908,17 @@
       <c r="F6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="4">
         <v>5</v>
       </c>
-      <c r="I6" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.84005428459187781</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K6" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.52802952345911347</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -901,15 +935,17 @@
       <c r="F7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="4">
         <v>6</v>
       </c>
-      <c r="I7" s="6">
-        <f ca="1">RAND()</f>
-        <v>2.7874064624666905E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K7" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.66633717432954598</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
@@ -926,15 +962,17 @@
       <c r="F8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="4">
         <v>7</v>
       </c>
-      <c r="I8" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.91536273521502443</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K8" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.49020863545915372</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -951,15 +989,17 @@
       <c r="F9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="4">
         <v>8</v>
       </c>
-      <c r="I9" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.71506805238535442</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K9" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.46504055343670092</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
         <v>30</v>
@@ -972,15 +1012,17 @@
       <c r="F10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="I10" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.29431600334252406</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K10" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.45454547228512554</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>34</v>
       </c>
@@ -995,16 +1037,18 @@
       <c r="F11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G11" s="4"/>
-      <c r="H11">
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="4"/>
+      <c r="J11">
         <v>1</v>
       </c>
-      <c r="I11" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.93016278882487313</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K11" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.23876680035666464</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>36</v>
       </c>
@@ -1019,16 +1063,18 @@
       <c r="F12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G12" s="4"/>
-      <c r="H12">
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="4"/>
+      <c r="J12">
         <v>4</v>
       </c>
-      <c r="I12" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.36342056568959991</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K12" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.65760833881478897</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>33</v>
       </c>
@@ -1043,16 +1089,18 @@
       <c r="F13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="4"/>
-      <c r="H13">
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="4"/>
+      <c r="J13">
         <v>2</v>
       </c>
-      <c r="I13" s="6">
-        <f ca="1">RAND()</f>
-        <v>7.8645057123848394E-3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="K13" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.94221376477563423</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
@@ -1067,13 +1115,15 @@
       <c r="F14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G14" s="4"/>
-      <c r="H14">
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="4"/>
+      <c r="J14">
         <v>3</v>
       </c>
-      <c r="I14" s="6">
-        <f ca="1">RAND()</f>
-        <v>0.61530357197018049</v>
+      <c r="K14" s="6">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.47763134536431928</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert project-specific ProjFiles attributes
</commit_message>
<xml_diff>
--- a/tests/test_data/ColInfo.xlsx
+++ b/tests/test_data/ColInfo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Library\CloudStorage\Box-Box\Projects\Excel_Steps\tests\test_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/j.d.landgrebe/Library/CloudStorage/Box-Box/Projects/Excel_Steps/tests/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93130DE0-5232-45EC-ADC1-180370F26015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D18F24C1-E0F3-7D45-A252-8050C6295B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="1905" windowWidth="26003" windowHeight="11535" xr2:uid="{CF177DA8-F40C-4AC0-BFD2-2712428C7C73}"/>
+    <workbookView xWindow="0" yWindow="1900" windowWidth="39260" windowHeight="20000" xr2:uid="{CF177DA8-F40C-4AC0-BFD2-2712428C7C73}"/>
   </bookViews>
   <sheets>
     <sheet name="colinfo_" sheetId="1" r:id="rId1"/>
@@ -730,21 +730,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D8961A3-90B8-45BB-ADA5-B09F327CFDF3}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.53125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.3984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.06640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.19921875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.796875" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
     <col min="9" max="9" width="10.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.73046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -779,7 +779,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -805,10 +805,10 @@
       </c>
       <c r="K2" s="6">
         <f t="shared" ref="K2:K14" ca="1" si="0">RAND()</f>
-        <v>0.10166470194637378</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+        <v>0.45378549633004195</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -834,10 +834,10 @@
       </c>
       <c r="K3" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.73948259909675951</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+        <v>0.44065664304530716</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -861,10 +861,10 @@
       </c>
       <c r="K4" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.53192412061943051</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+        <v>0.18291626723272969</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -888,10 +888,10 @@
       </c>
       <c r="K5" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>5.5982527382875014E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+        <v>7.7809451936697194E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -915,10 +915,10 @@
       </c>
       <c r="K6" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.40788799338347059</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+        <v>2.175374147656306E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -942,10 +942,10 @@
       </c>
       <c r="K7" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>3.2824126829218647E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+        <v>7.7120114445856647E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
@@ -969,10 +969,10 @@
       </c>
       <c r="K8" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.89047186805703138</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+        <v>0.32436105923441827</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -996,10 +996,10 @@
       </c>
       <c r="K9" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.5878531727357369</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+        <v>0.44988976626082122</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
         <v>30</v>
@@ -1019,10 +1019,10 @@
       </c>
       <c r="K10" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.5400778776490911</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+        <v>0.52053121433160321</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>34</v>
       </c>
@@ -1045,10 +1045,10 @@
       </c>
       <c r="K11" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.60171761733461671</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+        <v>0.82389445572818609</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>36</v>
       </c>
@@ -1071,10 +1071,10 @@
       </c>
       <c r="K12" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.92083275593773184</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+        <v>0.57383386483193588</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>33</v>
       </c>
@@ -1097,10 +1097,10 @@
       </c>
       <c r="K13" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.44994081162133492</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+        <v>0.52072799295753458</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
@@ -1123,7 +1123,7 @@
       </c>
       <c r="K14" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.43354329535425495</v>
+        <v>0.23517874195112898</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update tests based on recent changes --all pass except where noted in RunTests.bas comment
</commit_message>
<xml_diff>
--- a/tests/test_data/ColInfo.xlsx
+++ b/tests/test_data/ColInfo.xlsx
@@ -1,28 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/j.d.landgrebe/Library/CloudStorage/Box-Box/Projects/Excel_Steps/tests/test_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Library\CloudStorage\Box-Box\Projects\Excel_Steps\tests\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D18F24C1-E0F3-7D45-A252-8050C6295B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548C98EE-AA97-44F1-8A63-F0D945B6A6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1900" windowWidth="39260" windowHeight="20000" xr2:uid="{CF177DA8-F40C-4AC0-BFD2-2712428C7C73}"/>
+    <workbookView xWindow="1440" yWindow="1890" windowWidth="28800" windowHeight="11535" xr2:uid="{CF177DA8-F40C-4AC0-BFD2-2712428C7C73}"/>
   </bookViews>
   <sheets>
     <sheet name="colinfo_" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="BR_Example">colinfo_!$I:$I</definedName>
-    <definedName name="data_type_VBA">colinfo_!$F:$F</definedName>
-    <definedName name="Description">colinfo_!$D:$D</definedName>
-    <definedName name="IsIndex">colinfo_!$C:$C</definedName>
-    <definedName name="rand">colinfo_!$K:$K</definedName>
-    <definedName name="Second_Tbl">colinfo_!$J:$J</definedName>
-    <definedName name="units">colinfo_!$E:$E</definedName>
+    <definedName name="BR_Example">colinfo_!$J:$J</definedName>
+    <definedName name="data_type_VBA">colinfo_!$G:$G</definedName>
+    <definedName name="Description">colinfo_!$E:$E</definedName>
+    <definedName name="FillVals">colinfo_!$H:$H</definedName>
+    <definedName name="FilterVals">colinfo_!$I:$I</definedName>
+    <definedName name="IsIndex">colinfo_!$D:$D</definedName>
+    <definedName name="rand">colinfo_!$L:$L</definedName>
+    <definedName name="Second_Tbl">colinfo_!$K:$K</definedName>
+    <definedName name="units">colinfo_!$F:$F</definedName>
     <definedName name="VarNameNorm">colinfo_!$A:$A</definedName>
     <definedName name="VarNameRaw">colinfo_!$B:$B</definedName>
   </definedNames>
@@ -50,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
   <si>
     <t>Description</t>
   </si>
@@ -221,6 +223,21 @@
   </si>
   <si>
     <t>{KeepOnly:Online}</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>prodtype</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>serial_week</t>
   </si>
 </sst>
 </file>
@@ -729,22 +746,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D8961A3-90B8-45BB-ADA5-B09F327CFDF3}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L14"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.46484375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="4" max="4" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.796875" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -752,146 +770,161 @@
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="b">
+      <c r="C2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="2"/>
+      <c r="G2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="4">
+      <c r="J2" s="4">
         <v>1</v>
       </c>
-      <c r="K2" s="6">
-        <f t="shared" ref="K2:K14" ca="1" si="0">RAND()</f>
-        <v>0.45378549633004195</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" s="6">
+        <f t="shared" ref="L2:L14" ca="1" si="0">RAND()</f>
+        <v>0.2453989114435613</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="2" t="b">
+      <c r="C3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="2"/>
+      <c r="G3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="4">
+      <c r="I3" s="2"/>
+      <c r="J3" s="4">
         <v>2</v>
       </c>
-      <c r="K3" s="6">
+      <c r="L3" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.44065664304530716</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.86136552357971186</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="b">
+      <c r="C4" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="2"/>
+      <c r="G4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="2"/>
       <c r="H4" s="2"/>
-      <c r="I4" s="4">
+      <c r="I4" s="2"/>
+      <c r="J4" s="4">
         <v>3</v>
       </c>
-      <c r="K4" s="6">
+      <c r="L4" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.18291626723272969</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+        <v>3.1813151983975274E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="2" t="b">
+      <c r="C5" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="2"/>
+      <c r="G5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="2"/>
       <c r="H5" s="2"/>
-      <c r="I5" s="4">
+      <c r="I5" s="2"/>
+      <c r="J5" s="4">
         <v>4</v>
       </c>
-      <c r="K5" s="6">
+      <c r="L5" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>7.7809451936697194E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.32245624498281522</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -899,26 +932,27 @@
         <v>17</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="2"/>
+      <c r="E6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="4">
+      <c r="I6" s="2"/>
+      <c r="J6" s="4">
         <v>5</v>
       </c>
-      <c r="K6" s="6">
+      <c r="L6" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>2.175374147656306E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.87170413600850527</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -926,26 +960,27 @@
         <v>18</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="2"/>
+      <c r="E7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="4">
+      <c r="I7" s="2"/>
+      <c r="J7" s="4">
         <v>6</v>
       </c>
-      <c r="K7" s="6">
+      <c r="L7" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>7.7120114445856647E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.53010823770860449</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
@@ -953,26 +988,27 @@
         <v>19</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="2"/>
+      <c r="E8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="2"/>
       <c r="H8" s="2"/>
-      <c r="I8" s="4">
+      <c r="I8" s="2"/>
+      <c r="J8" s="4">
         <v>7</v>
       </c>
-      <c r="K8" s="6">
+      <c r="L8" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.32436105923441827</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.75538465633279606</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -980,49 +1016,51 @@
         <v>20</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="2"/>
+      <c r="E9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="4">
+      <c r="I9" s="2"/>
+      <c r="J9" s="4">
         <v>8</v>
       </c>
-      <c r="K9" s="6">
+      <c r="L9" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.44988976626082122</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.42879314574025174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
         <v>30</v>
       </c>
       <c r="C10" s="2"/>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="2"/>
+      <c r="E10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="2"/>
+      <c r="G10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="2"/>
+      <c r="J10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K10" s="6">
+      <c r="L10" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.52053121433160321</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.59303248016299559</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>34</v>
       </c>
@@ -1030,25 +1068,26 @@
         <v>38</v>
       </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="3"/>
+      <c r="E11" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="3"/>
+      <c r="G11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G11" s="3"/>
       <c r="H11" s="3"/>
-      <c r="I11" s="4"/>
-      <c r="J11">
+      <c r="I11" s="3"/>
+      <c r="J11" s="4"/>
+      <c r="K11">
         <v>1</v>
       </c>
-      <c r="K11" s="6">
+      <c r="L11" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.82389445572818609</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.63878754852183117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>36</v>
       </c>
@@ -1056,25 +1095,26 @@
         <v>41</v>
       </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="3"/>
+      <c r="E12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="3"/>
+      <c r="G12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G12" s="3"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="4"/>
-      <c r="J12">
+      <c r="I12" s="3"/>
+      <c r="J12" s="4"/>
+      <c r="K12">
         <v>4</v>
       </c>
-      <c r="K12" s="6">
+      <c r="L12" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.57383386483193588</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.83569582663199538</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>33</v>
       </c>
@@ -1082,25 +1122,26 @@
         <v>39</v>
       </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="3"/>
+      <c r="E13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="3"/>
+      <c r="G13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="3"/>
       <c r="H13" s="3"/>
-      <c r="I13" s="4"/>
-      <c r="J13">
+      <c r="I13" s="3"/>
+      <c r="J13" s="4"/>
+      <c r="K13">
         <v>2</v>
       </c>
-      <c r="K13" s="6">
+      <c r="L13" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.52072799295753458</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0.60669556748942988</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
@@ -1108,22 +1149,23 @@
         <v>40</v>
       </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="3"/>
+      <c r="E14" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="3"/>
+      <c r="G14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G14" s="3"/>
       <c r="H14" s="3"/>
-      <c r="I14" s="4"/>
-      <c r="J14">
+      <c r="I14" s="3"/>
+      <c r="J14" s="4"/>
+      <c r="K14">
         <v>3</v>
       </c>
-      <c r="K14" s="6">
+      <c r="L14" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>0.23517874195112898</v>
+        <v>5.4306262047155052E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>